<commit_message>
Fix watershed over-split of elongated lacunae (generalized to N pieces)
merge_shallow_splits() in segment_lacunae_v2.py: first version only
handled the exactly-2-substantial-pieces case and missed a case with 3
raw pieces (2 kept + 1 rejected by shape filters). Generalized to
union-find over pairwise shallow-saddle links, so any chain of shallow
splits within one pre-watershed component merges correctly.

Verified via src/diagnose_lacuna_splits.py: 12 candidate 2-piece splits
across all 8 WT images down to 1 (682_z29c1-3 component 174, ratio 0.000
-- a genuine two-lobe separation, correctly left split). All 3 splits the
user confirmed as wrong by eye (542 WT 2_z06c1-2) are now merged; verified
visually on that image's overlay too (every lacuna now one clean outline).

results/count/ and results/canaliculi/ regenerated against the fix.
PROGRESS.md updated: issue marked resolved with the verified numbers.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/canaliculi/542_WT__2_z06c1-2/measurements.xlsx
+++ b/results/canaliculi/542_WT__2_z06c1-2/measurements.xlsx
@@ -441,10 +441,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -493,13 +493,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30.6471</v>
+        <v>37.6154</v>
       </c>
       <c r="C6" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="D6" t="n">
-        <v>22.3017</v>
+        <v>21.5853</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -517,13 +517,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>137.8234</v>
+        <v>157.0446</v>
       </c>
       <c r="C7" t="n">
-        <v>126.1006</v>
+        <v>147.2442</v>
       </c>
       <c r="D7" t="n">
-        <v>61.6695</v>
+        <v>60.263</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -717,13 +717,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C8" t="n">
-        <v>1639.3078</v>
+        <v>1995.984</v>
       </c>
       <c r="D8" t="n">
-        <v>126.1006</v>
+        <v>90.7265</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -739,13 +739,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C9" t="n">
-        <v>1410.3128</v>
+        <v>3491.64</v>
       </c>
       <c r="D9" t="n">
-        <v>74.227</v>
+        <v>166.2686</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -761,13 +761,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="C10" t="n">
-        <v>1995.984</v>
+        <v>12899.4022</v>
       </c>
       <c r="D10" t="n">
-        <v>90.7265</v>
+        <v>204.7524</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -783,13 +783,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="C11" t="n">
-        <v>1629.4794</v>
+        <v>3059.8805</v>
       </c>
       <c r="D11" t="n">
-        <v>135.7899</v>
+        <v>95.62130000000001</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -805,13 +805,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="C12" t="n">
-        <v>501.6173</v>
+        <v>27966.6009</v>
       </c>
       <c r="D12" t="n">
-        <v>45.6016</v>
+        <v>285.3735</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -827,13 +827,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="C13" t="n">
-        <v>12899.4022</v>
+        <v>5006.304</v>
       </c>
       <c r="D13" t="n">
-        <v>204.7524</v>
+        <v>147.2442</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -849,13 +849,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C14" t="n">
-        <v>3058.4663</v>
+        <v>3505.5395</v>
       </c>
       <c r="D14" t="n">
-        <v>95.5771</v>
+        <v>100.1583</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -871,13 +871,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>98</v>
+        <v>28</v>
       </c>
       <c r="C15" t="n">
-        <v>27966.6009</v>
+        <v>4289.5365</v>
       </c>
       <c r="D15" t="n">
-        <v>285.3735</v>
+        <v>153.1977</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -893,16 +893,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="C16" t="n">
-        <v>5006.304</v>
+        <v>3917.2014</v>
       </c>
       <c r="D16" t="n">
-        <v>147.2442</v>
+        <v>244.8251</v>
       </c>
       <c r="E16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -915,106 +915,18 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C17" t="n">
-        <v>3505.5395</v>
+        <v>9071.2425</v>
       </c>
       <c r="D17" t="n">
-        <v>100.1583</v>
+        <v>201.5832</v>
       </c>
       <c r="E17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="inlineStr">
-        <is>
-          <t>px</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" t="n">
-        <v>9</v>
-      </c>
-      <c r="C18" t="n">
-        <v>1155.5778</v>
-      </c>
-      <c r="D18" t="n">
-        <v>128.3975</v>
-      </c>
-      <c r="E18" t="b">
-        <v>0</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>px</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" t="n">
-        <v>17</v>
-      </c>
-      <c r="C19" t="n">
-        <v>1883.8002</v>
-      </c>
-      <c r="D19" t="n">
-        <v>110.8118</v>
-      </c>
-      <c r="E19" t="b">
-        <v>0</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>px</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" t="n">
-        <v>16</v>
-      </c>
-      <c r="C20" t="n">
-        <v>3917.2014</v>
-      </c>
-      <c r="D20" t="n">
-        <v>244.8251</v>
-      </c>
-      <c r="E20" t="b">
-        <v>1</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>px</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" t="n">
-        <v>45</v>
-      </c>
-      <c r="C21" t="n">
-        <v>9071.2425</v>
-      </c>
-      <c r="D21" t="n">
-        <v>201.5832</v>
-      </c>
-      <c r="E21" t="b">
-        <v>1</v>
-      </c>
-      <c r="F21" t="inlineStr">
         <is>
           <t>px</t>
         </is>

</xml_diff>

<commit_message>
Regenerate stale default canaliculi outputs for 7 WT images
The top-level default outputs in results/canaliculi/<image>/ for every
image except 543-2 were last written on 2026-09-22, before hysteresis,
gap bridging and BLOCK_GROWTH_IN_FLAGGED existed (their JSON has no
threshold_mode key). Only 543-2 had been regenerated, as the reference
check. This rewrites them with the current defaults and adds the
bridges.png each default run now produces. No code change.

Mean edge count per cell, old file to current default:
542_z06 20.15 to 30.85, 543_3 23.78 to 47.11, 682_z29 13.55 to 26.18.
543-2 unchanged at 62.33 / 27.41.

Pre-validation, pixel units.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/canaliculi/542_WT__2_z06c1-2/measurements.xlsx
+++ b/results/canaliculi/542_WT__2_z06c1-2/measurements.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="per_lacuna" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="field" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="per_lacuna" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -530,13 +531,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20.1538</v>
+        <v>30.8462</v>
       </c>
       <c r="C7" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D7" t="n">
-        <v>12.0267</v>
+        <v>21.0113</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -554,13 +555,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>664.9475</v>
+        <v>988.2809</v>
       </c>
       <c r="C8" t="n">
-        <v>495.5879</v>
+        <v>919.2935</v>
       </c>
       <c r="D8" t="n">
-        <v>416.4797</v>
+        <v>748.3807</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -578,13 +579,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>32.4293</v>
+        <v>31.5991</v>
       </c>
       <c r="C9" t="n">
-        <v>32.9674</v>
+        <v>33.5078</v>
       </c>
       <c r="D9" t="n">
-        <v>7.8559</v>
+        <v>7.5869</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -606,6 +607,206 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>per-field metrics -- independent of the per-lacuna assignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Only ~23% of skeleton length is graph-connected to any lacuna in these 2D</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>sections, so per-cell numbers use a quarter of the network. These use all of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>analysed_area_px2</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1009061</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>total_skeleton_length_px</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>34964</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>canalicular_length_density_per_px</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.03465004</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>px^-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>junction_count</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>375</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>junction_density_per_px2</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.00037163</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>px^-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>lacuna_count</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>16</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>lacunae_per_px2</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1.586e-05</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>px^-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>skeleton_component_count</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>654</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>mean_component_length_px</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>53.4618</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>median_component_length_px</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>23</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -646,13 +847,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C2" t="n">
-        <v>903.394</v>
+        <v>1032.992</v>
       </c>
       <c r="D2" t="n">
-        <v>37.6414</v>
+        <v>31.3028</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -671,10 +872,10 @@
         <v>10</v>
       </c>
       <c r="C3" t="n">
-        <v>329.5929</v>
+        <v>335.0782</v>
       </c>
       <c r="D3" t="n">
-        <v>32.9593</v>
+        <v>33.5078</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -690,13 +891,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>267.2792</v>
+        <v>292.9361</v>
       </c>
       <c r="D4" t="n">
-        <v>24.2981</v>
+        <v>19.5291</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -712,13 +913,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C5" t="n">
-        <v>129.397</v>
+        <v>387.1909</v>
       </c>
       <c r="D5" t="n">
-        <v>18.4853</v>
+        <v>27.6565</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -734,13 +935,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>428.5757</v>
+        <v>504.931</v>
       </c>
       <c r="D6" t="n">
-        <v>32.9674</v>
+        <v>33.6621</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -756,13 +957,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C7" t="n">
-        <v>1224.3301</v>
+        <v>1337.6144</v>
       </c>
       <c r="D7" t="n">
-        <v>31.3931</v>
+        <v>28.4599</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -778,13 +979,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C8" t="n">
-        <v>543.7178</v>
+        <v>688.6589</v>
       </c>
       <c r="D8" t="n">
-        <v>38.837</v>
+        <v>36.2452</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -800,13 +1001,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C9" t="n">
-        <v>364.664</v>
+        <v>414.1198</v>
       </c>
       <c r="D9" t="n">
-        <v>21.4508</v>
+        <v>20.706</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -822,13 +1023,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="C10" t="n">
-        <v>495.5879</v>
+        <v>1157.4012</v>
       </c>
       <c r="D10" t="n">
-        <v>35.3991</v>
+        <v>35.0728</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -844,13 +1045,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C11" t="n">
-        <v>969.9626</v>
+        <v>919.2935</v>
       </c>
       <c r="D11" t="n">
-        <v>44.0892</v>
+        <v>45.9647</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -866,13 +1067,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C12" t="n">
-        <v>1487.3372</v>
+        <v>1771.6043</v>
       </c>
       <c r="D12" t="n">
-        <v>34.5892</v>
+        <v>32.211</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -888,13 +1089,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C13" t="n">
-        <v>943.796</v>
+        <v>955.2397</v>
       </c>
       <c r="D13" t="n">
-        <v>26.2166</v>
+        <v>22.7438</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -910,13 +1111,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>25</v>
+        <v>83</v>
       </c>
       <c r="C14" t="n">
-        <v>1018.2468</v>
+        <v>2992.182</v>
       </c>
       <c r="D14" t="n">
-        <v>40.7299</v>
+        <v>36.0504</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -932,13 +1133,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="C15" t="n">
-        <v>441.8305</v>
+        <v>1091.4012</v>
       </c>
       <c r="D15" t="n">
-        <v>40.1664</v>
+        <v>38.9786</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -954,13 +1155,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C16" t="n">
-        <v>298.0366</v>
+        <v>404.3919</v>
       </c>
       <c r="D16" t="n">
-        <v>18.6273</v>
+        <v>20.2196</v>
       </c>
       <c r="E16" t="b">
         <v>1</v>
@@ -976,13 +1177,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C17" t="n">
-        <v>57.6274</v>
+        <v>97.08329999999999</v>
       </c>
       <c r="D17" t="n">
-        <v>19.2091</v>
+        <v>16.1805</v>
       </c>
       <c r="E17" t="b">
         <v>1</v>

</xml_diff>